<commit_message>
revert harga_pangan db dependency, source prices from Sagon, route stunting/SKPG tables, update header texts and production labels
</commit_message>
<xml_diff>
--- a/public/template_gizi_balita.xlsx
+++ b/public/template_gizi_balita.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,18 +407,21 @@
         <v>Bulan</v>
       </c>
       <c r="C1" t="str">
+        <v>Kecamatan</v>
+      </c>
+      <c r="D1" t="str">
         <v>nama_kelurahan</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>gizi_sangat_kurang</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>gizi_kurang</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>gizi_normal</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>gizi_berlebih</v>
       </c>
     </row>
@@ -430,18 +433,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="str">
+        <v>Cilegon</v>
+      </c>
+      <c r="D2" t="str">
         <v>Bagendung</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>10</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>23</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>673</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>27</v>
       </c>
     </row>
@@ -453,24 +459,27 @@
         <v>1</v>
       </c>
       <c r="C3" t="str">
+        <v>Ciwandan</v>
+      </c>
+      <c r="D3" t="str">
         <v>Banjar Negara</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>17</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>70</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>553</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>12</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>